<commit_message>
docs: record final dense-range optimization and acceptance results
</commit_message>
<xml_diff>
--- a/tests/ExcelRenderer.Formulas.Tests/Fixtures/Oracle/Mapping/mapping-0.xlsx
+++ b/tests/ExcelRenderer.Formulas.Tests/Fixtures/Oracle/Mapping/mapping-0.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice" sheetId="1" r:id="R7b82c7eab7ad4529"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rates" sheetId="2" r:id="R571af047bc06445f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="3" r:id="R3b4edb28181144d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice" sheetId="1" r:id="Rf061f61826fb4a11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rates" sheetId="2" r:id="R242b85fc07ad4319"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="3" r:id="Rcd5b3a1b982a4634"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="Amounts">'Invoice'!$D$1:$D$1</x:definedName>

</xml_diff>